<commit_message>
filled out schedule - first pass
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="64">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -34,7 +34,7 @@
     <t xml:space="preserve">Section</t>
   </si>
   <si>
-    <t xml:space="preserve">Notes</t>
+    <t xml:space="preserve">Additional Topics / Notes</t>
   </si>
   <si>
     <t xml:space="preserve">F</t>
@@ -67,51 +67,163 @@
     <t xml:space="preserve">Linear Algebra</t>
   </si>
   <si>
+    <t xml:space="preserve">First application of time complexity analysis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gaussian Elimination</t>
+  </si>
+  <si>
     <t xml:space="preserve">Lab 1: Solving Linear Systems</t>
   </si>
   <si>
+    <t xml:space="preserve">A bad algorithm: Cramer’s Method</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analysis of recursive algorithms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LU Factorization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Numerical Stability, Matrix Condition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bracketing Methods</t>
+  </si>
+  <si>
     <t xml:space="preserve">Nonlinear Algebraic Equations</t>
   </si>
   <si>
+    <t xml:space="preserve">Fixed Point Iteration</t>
+  </si>
+  <si>
     <t xml:space="preserve">Lab 2: Solving Nonlinear Systems</t>
   </si>
   <si>
+    <t xml:space="preserve">Newton’s Method</t>
+  </si>
+  <si>
     <t xml:space="preserve">Modeling</t>
   </si>
   <si>
     <t xml:space="preserve">Code Interview 1</t>
   </si>
   <si>
+    <t xml:space="preserve">Euler’s Method</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ordinary Differential Equations</t>
   </si>
   <si>
+    <t xml:space="preserve">Also, exact solutions to linear </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Runge-Kutta Methods</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Including adaptive Runge-Kutta</t>
+  </si>
+  <si>
     <t xml:space="preserve">Lab 3: Simulating ODEs</t>
   </si>
   <si>
+    <t xml:space="preserve">Stiff equations and Implicit integration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boundary Value: Shooting and Finite Difference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Review?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exam 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probably move this earlier!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unconstrained Optimization Problems</t>
+  </si>
+  <si>
     <t xml:space="preserve">Optimization</t>
   </si>
   <si>
-    <t xml:space="preserve">Exam 1</t>
+    <t xml:space="preserve">Should be Review, Necessary and sufficient conditions for optimality</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gradient Descent</t>
   </si>
   <si>
     <t xml:space="preserve">Lab 4: Optimization</t>
   </si>
   <si>
+    <t xml:space="preserve">Line Search, Momentum, ADAM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maybe also touch on Quasi-Newton/Conjugate Gradient</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Constrained Optimization: Lagrange Multipliers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neither book talks about constraints</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interior point methods</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Could alternatively do Augmented Lagrangian, but I think interior point has the best </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regression problems and least-squares</t>
+  </si>
+  <si>
     <t xml:space="preserve">Regression and Learning</t>
   </si>
   <si>
+    <t xml:space="preserve">R-squared value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Least-squares with nonlinear basis functions</t>
+  </si>
+  <si>
     <t xml:space="preserve">Lab 5: Regression</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neural Networks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Limit to MLPs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gradients of Neural Network Parameters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stochastic Gradient Descent / Stochastic ADAM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Training Neural Networks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Including some form of regularization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Final Exam Slot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exam 2?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
+    <numFmt numFmtId="166" formatCode="mm/dd/yy"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -149,6 +261,21 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFC9211E"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -159,32 +286,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF92E285"/>
-        <bgColor rgb="FF99CCFF"/>
+        <fgColor rgb="FFA5D6A7"/>
+        <bgColor rgb="FF90CAF9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF63BBEE"/>
-        <bgColor rgb="FF99CCFF"/>
+        <fgColor rgb="FF90CAF9"/>
+        <bgColor rgb="FFA5D6A7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF09E6F"/>
-        <bgColor rgb="FFFF99CC"/>
+        <fgColor rgb="FFFFAB91"/>
+        <bgColor rgb="FFFFCC99"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFDC85E9"/>
-        <bgColor rgb="FFFF99CC"/>
+        <fgColor rgb="FFCE93D8"/>
+        <bgColor rgb="FF9999FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF5CD53"/>
-        <bgColor rgb="FFFFCC00"/>
+        <fgColor rgb="FFFFF59D"/>
+        <bgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -222,7 +349,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -271,6 +398,14 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -279,11 +414,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -321,14 +460,14 @@
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FF92E285"/>
+      <rgbColor rgb="FFA5D6A7"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFFFFCC"/>
       <rgbColor rgb="FFDCE6F1"/>
       <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFF09E6F"/>
+      <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
       <rgbColor rgb="FFCCCCFF"/>
       <rgbColor rgb="FF000080"/>
@@ -342,13 +481,13 @@
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFFF99"/>
-      <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FFDC85E9"/>
-      <rgbColor rgb="FFF5CD53"/>
+      <rgbColor rgb="FFFFF59D"/>
+      <rgbColor rgb="FF90CAF9"/>
+      <rgbColor rgb="FFFFAB91"/>
+      <rgbColor rgb="FFCE93D8"/>
+      <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
-      <rgbColor rgb="FF63BBEE"/>
+      <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
@@ -359,7 +498,7 @@
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FFC9211E"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
@@ -548,12 +687,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="43.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="30"/>
   </cols>
   <sheetData>
@@ -641,7 +780,9 @@
       <c r="D6" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="4"/>
+      <c r="E6" s="4" t="s">
+        <v>15</v>
+      </c>
       <c r="F6" s="4"/>
     </row>
     <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -651,7 +792,9 @@
       <c r="B7" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="4"/>
+      <c r="C7" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="D7" s="7"/>
       <c r="E7" s="4"/>
     </row>
@@ -663,7 +806,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D8" s="7"/>
       <c r="E8" s="4"/>
@@ -675,9 +818,13 @@
       <c r="B9" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="4"/>
+      <c r="C9" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="D9" s="7"/>
-      <c r="E9" s="4"/>
+      <c r="E9" s="4" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="n">
@@ -686,9 +833,13 @@
       <c r="B10" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="4"/>
+      <c r="C10" s="4" t="s">
+        <v>20</v>
+      </c>
       <c r="D10" s="7"/>
-      <c r="E10" s="4"/>
+      <c r="E10" s="4" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="n">
@@ -698,7 +849,7 @@
         <v>5</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D11" s="7"/>
       <c r="E11" s="4"/>
@@ -710,9 +861,11 @@
       <c r="B12" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="4"/>
+      <c r="C12" s="4" t="s">
+        <v>22</v>
+      </c>
       <c r="D12" s="8" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="E12" s="4"/>
     </row>
@@ -723,7 +876,9 @@
       <c r="B13" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="4"/>
+      <c r="C13" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="D13" s="9"/>
       <c r="E13" s="4"/>
     </row>
@@ -735,7 +890,7 @@
         <v>5</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="D14" s="9"/>
       <c r="E14" s="4"/>
@@ -747,7 +902,9 @@
       <c r="B15" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="4"/>
+      <c r="C15" s="4" t="s">
+        <v>26</v>
+      </c>
       <c r="D15" s="9"/>
       <c r="E15" s="4"/>
     </row>
@@ -770,7 +927,7 @@
         <v>5</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="D17" s="9"/>
       <c r="E17" s="4"/>
@@ -784,7 +941,7 @@
       </c>
       <c r="C18" s="4"/>
       <c r="D18" s="4" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="E18" s="4"/>
     </row>
@@ -807,7 +964,7 @@
         <v>5</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
@@ -819,11 +976,15 @@
       <c r="B21" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C21" s="4"/>
+      <c r="C21" s="4" t="s">
+        <v>29</v>
+      </c>
       <c r="D21" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E21" s="4"/>
+        <v>30</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="n">
@@ -832,9 +993,13 @@
       <c r="B22" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C22" s="4"/>
+      <c r="C22" s="4" t="s">
+        <v>32</v>
+      </c>
       <c r="D22" s="11"/>
-      <c r="E22" s="4"/>
+      <c r="E22" s="4" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="n">
@@ -844,7 +1009,7 @@
         <v>5</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="D23" s="11"/>
       <c r="E23" s="4"/>
@@ -856,7 +1021,9 @@
       <c r="B24" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C24" s="4"/>
+      <c r="C24" s="0" t="s">
+        <v>35</v>
+      </c>
       <c r="D24" s="11"/>
       <c r="E24" s="4"/>
     </row>
@@ -867,7 +1034,9 @@
       <c r="B25" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C25" s="4"/>
+      <c r="C25" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="D25" s="11"/>
       <c r="E25" s="4"/>
     </row>
@@ -879,7 +1048,7 @@
         <v>5</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="D26" s="11"/>
       <c r="E26" s="4"/>
@@ -891,10 +1060,10 @@
       <c r="B27" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C27" s="4"/>
-      <c r="D27" s="12" t="s">
-        <v>22</v>
-      </c>
+      <c r="C27" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D27" s="12"/>
       <c r="E27" s="4"/>
     </row>
     <row r="28" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -905,9 +1074,11 @@
         <v>10</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D28" s="13"/>
+        <v>38</v>
+      </c>
+      <c r="D28" s="13" t="s">
+        <v>39</v>
+      </c>
       <c r="E28" s="4"/>
     </row>
     <row r="29" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -918,7 +1089,7 @@
         <v>5</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="D29" s="13"/>
       <c r="E29" s="4"/>
@@ -930,9 +1101,15 @@
       <c r="B30" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C30" s="4"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="4"/>
+      <c r="C30" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="n">
@@ -941,8 +1118,10 @@
       <c r="B31" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C31" s="4"/>
-      <c r="D31" s="13"/>
+      <c r="C31" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31" s="15"/>
       <c r="E31" s="4"/>
     </row>
     <row r="32" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -953,9 +1132,9 @@
         <v>5</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="D32" s="13"/>
+        <v>44</v>
+      </c>
+      <c r="D32" s="15"/>
       <c r="E32" s="4"/>
     </row>
     <row r="33" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -965,9 +1144,11 @@
       <c r="B33" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C33" s="4"/>
-      <c r="D33" s="13"/>
-      <c r="E33" s="4"/>
+      <c r="C33" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D33" s="15"/>
+      <c r="E33" s="0"/>
     </row>
     <row r="34" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="n">
@@ -976,9 +1157,13 @@
       <c r="B34" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C34" s="4"/>
-      <c r="D34" s="13"/>
-      <c r="E34" s="4"/>
+      <c r="C34" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D34" s="15"/>
+      <c r="E34" s="4" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="n">
@@ -988,9 +1173,9 @@
         <v>5</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="D35" s="13"/>
+        <v>44</v>
+      </c>
+      <c r="D35" s="15"/>
       <c r="E35" s="4"/>
     </row>
     <row r="36" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1000,11 +1185,13 @@
       <c r="B36" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C36" s="4"/>
-      <c r="D36" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="E36" s="4"/>
+      <c r="C36" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D36" s="15"/>
+      <c r="E36" s="4" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="n">
@@ -1013,9 +1200,13 @@
       <c r="B37" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C37" s="4"/>
+      <c r="C37" s="4" t="s">
+        <v>49</v>
+      </c>
       <c r="D37" s="15"/>
-      <c r="E37" s="4"/>
+      <c r="E37" s="4" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="n">
@@ -1025,7 +1216,7 @@
         <v>5</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="D38" s="15"/>
       <c r="E38" s="4"/>
@@ -1037,9 +1228,15 @@
       <c r="B39" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C39" s="4"/>
-      <c r="D39" s="15"/>
-      <c r="E39" s="4"/>
+      <c r="C39" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D39" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="n">
@@ -1048,8 +1245,10 @@
       <c r="B40" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C40" s="4"/>
-      <c r="D40" s="15"/>
+      <c r="C40" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D40" s="17"/>
       <c r="E40" s="4"/>
     </row>
     <row r="41" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1060,9 +1259,9 @@
         <v>5</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D41" s="15"/>
+        <v>55</v>
+      </c>
+      <c r="D41" s="17"/>
       <c r="E41" s="4"/>
     </row>
     <row r="42" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1072,9 +1271,13 @@
       <c r="B42" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C42" s="4"/>
-      <c r="D42" s="15"/>
-      <c r="E42" s="4"/>
+      <c r="C42" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D42" s="17"/>
+      <c r="E42" s="4" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="n">
@@ -1083,8 +1286,10 @@
       <c r="B43" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C43" s="4"/>
-      <c r="D43" s="15"/>
+      <c r="C43" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D43" s="17"/>
       <c r="E43" s="4"/>
     </row>
     <row r="44" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1095,9 +1300,9 @@
         <v>5</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D44" s="15"/>
+        <v>55</v>
+      </c>
+      <c r="D44" s="17"/>
       <c r="E44" s="4"/>
     </row>
     <row r="45" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1107,8 +1312,10 @@
       <c r="B45" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C45" s="4"/>
-      <c r="D45" s="0"/>
+      <c r="C45" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D45" s="17"/>
       <c r="E45" s="4"/>
     </row>
     <row r="46" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1118,9 +1325,13 @@
       <c r="B46" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C46" s="4"/>
-      <c r="D46" s="0"/>
-      <c r="E46" s="4"/>
+      <c r="C46" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D46" s="17"/>
+      <c r="E46" s="4" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="n">
@@ -1129,19 +1340,35 @@
       <c r="B47" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C47" s="4"/>
-      <c r="D47" s="0"/>
+      <c r="C47" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D47" s="17"/>
       <c r="E47" s="4"/>
     </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="18" t="n">
+        <v>46365</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:B47 C39:C47 C2:C37">
+  <conditionalFormatting sqref="A2:B47 C23 C2:C21 E22 C31:C47 C25:C29">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>$B2="F"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C38">
+  <conditionalFormatting sqref="C22">
     <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>$B38="F"</formula>
+      <formula>$B22="F"</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
added a few things after thinking
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="63">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -49,7 +49,7 @@
     <t xml:space="preserve">Intro</t>
   </si>
   <si>
-    <t xml:space="preserve">AMVF Framework</t>
+    <t xml:space="preserve">AMVF Framework, Engineering with and without AI</t>
   </si>
   <si>
     <t xml:space="preserve">W</t>
@@ -103,7 +103,7 @@
     <t xml:space="preserve">Newton’s Method</t>
   </si>
   <si>
-    <t xml:space="preserve">Modeling</t>
+    <t xml:space="preserve">Exam 1</t>
   </si>
   <si>
     <t xml:space="preserve">Code Interview 1</t>
@@ -133,15 +133,6 @@
     <t xml:space="preserve">Boundary Value: Shooting and Finite Difference</t>
   </si>
   <si>
-    <t xml:space="preserve">Review?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exam 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Probably move this earlier!</t>
-  </si>
-  <si>
     <t xml:space="preserve">Unconstrained Optimization Problems</t>
   </si>
   <si>
@@ -154,12 +145,12 @@
     <t xml:space="preserve">Gradient Descent</t>
   </si>
   <si>
+    <t xml:space="preserve">Line Search, Momentum, ADAM</t>
+  </si>
+  <si>
     <t xml:space="preserve">Lab 4: Optimization</t>
   </si>
   <si>
-    <t xml:space="preserve">Line Search, Momentum, ADAM</t>
-  </si>
-  <si>
     <t xml:space="preserve">Maybe also touch on Quasi-Newton/Conjugate Gradient</t>
   </si>
   <si>
@@ -175,6 +166,9 @@
     <t xml:space="preserve">Could alternatively do Augmented Lagrangian, but I think interior point has the best </t>
   </si>
   <si>
+    <t xml:space="preserve">Exam 2</t>
+  </si>
+  <si>
     <t xml:space="preserve">Regression problems and least-squares</t>
   </si>
   <si>
@@ -199,6 +193,9 @@
     <t xml:space="preserve">Gradients of Neural Network Parameters</t>
   </si>
   <si>
+    <t xml:space="preserve">THANKSGIVING BREAK</t>
+  </si>
+  <si>
     <t xml:space="preserve">Stochastic Gradient Descent / Stochastic ADAM</t>
   </si>
   <si>
@@ -211,7 +208,7 @@
     <t xml:space="preserve">Final Exam Slot</t>
   </si>
   <si>
-    <t xml:space="preserve">Exam 2?</t>
+    <t xml:space="preserve">Final Exam</t>
   </si>
 </sst>
 </file>
@@ -349,7 +346,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -398,11 +395,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -692,7 +685,7 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="43.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="43.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="30"/>
   </cols>
   <sheetData>
@@ -939,10 +932,10 @@
       <c r="B18" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4" t="s">
+      <c r="C18" s="4" t="s">
         <v>27</v>
       </c>
+      <c r="D18" s="4"/>
       <c r="E18" s="4"/>
     </row>
     <row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1021,7 +1014,7 @@
       <c r="B24" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C24" s="0" t="s">
+      <c r="C24" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D24" s="11"/>
@@ -1060,9 +1053,7 @@
       <c r="B27" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C27" s="4" t="s">
-        <v>37</v>
-      </c>
+      <c r="C27" s="4"/>
       <c r="D27" s="12"/>
       <c r="E27" s="4"/>
     </row>
@@ -1073,13 +1064,15 @@
       <c r="B28" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D28" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="D28" s="13" t="s">
+      <c r="E28" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E28" s="4"/>
     </row>
     <row r="29" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="n">
@@ -1091,7 +1084,7 @@
       <c r="C29" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D29" s="13"/>
+      <c r="D29" s="14"/>
       <c r="E29" s="4"/>
     </row>
     <row r="30" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1101,15 +1094,11 @@
       <c r="B30" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C30" s="0" t="s">
+      <c r="C30" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D30" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="E30" s="4" t="s">
-        <v>42</v>
-      </c>
+      <c r="D30" s="14"/>
+      <c r="E30" s="4"/>
     </row>
     <row r="31" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="n">
@@ -1119,10 +1108,9 @@
         <v>10</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D31" s="15"/>
-      <c r="E31" s="4"/>
+        <v>41</v>
+      </c>
+      <c r="D31" s="14"/>
     </row>
     <row r="32" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="n">
@@ -1132,10 +1120,9 @@
         <v>5</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="D32" s="15"/>
-      <c r="E32" s="4"/>
+        <v>42</v>
+      </c>
+      <c r="D32" s="14"/>
     </row>
     <row r="33" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="n">
@@ -1145,10 +1132,12 @@
         <v>7</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="D33" s="15"/>
-      <c r="E33" s="0"/>
+        <v>26</v>
+      </c>
+      <c r="D33" s="14"/>
+      <c r="E33" s="4" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="n">
@@ -1158,11 +1147,11 @@
         <v>10</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D34" s="15"/>
+        <v>44</v>
+      </c>
+      <c r="D34" s="14"/>
       <c r="E34" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1173,10 +1162,9 @@
         <v>5</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="D35" s="15"/>
-      <c r="E35" s="4"/>
+        <v>42</v>
+      </c>
+      <c r="D35" s="14"/>
     </row>
     <row r="36" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="n">
@@ -1186,11 +1174,11 @@
         <v>7</v>
       </c>
       <c r="C36" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D36" s="14"/>
+      <c r="E36" s="4" t="s">
         <v>47</v>
-      </c>
-      <c r="D36" s="15"/>
-      <c r="E36" s="4" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1200,12 +1188,8 @@
       <c r="B37" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C37" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="D37" s="15"/>
-      <c r="E37" s="4" t="s">
-        <v>50</v>
+      <c r="C37" s="1" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1216,9 +1200,8 @@
         <v>5</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="D38" s="15"/>
+        <v>42</v>
+      </c>
       <c r="E38" s="4"/>
     </row>
     <row r="39" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1229,13 +1212,13 @@
         <v>7</v>
       </c>
       <c r="C39" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D39" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="E39" s="4" t="s">
         <v>51</v>
-      </c>
-      <c r="D39" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="E39" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1246,9 +1229,9 @@
         <v>10</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="D40" s="17"/>
+        <v>52</v>
+      </c>
+      <c r="D40" s="16"/>
       <c r="E40" s="4"/>
     </row>
     <row r="41" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1259,9 +1242,9 @@
         <v>5</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D41" s="17"/>
+        <v>53</v>
+      </c>
+      <c r="D41" s="16"/>
       <c r="E41" s="4"/>
     </row>
     <row r="42" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1272,11 +1255,11 @@
         <v>7</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="D42" s="17"/>
+        <v>54</v>
+      </c>
+      <c r="D42" s="16"/>
       <c r="E42" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1287,9 +1270,9 @@
         <v>10</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="D43" s="17"/>
+        <v>56</v>
+      </c>
+      <c r="D43" s="16"/>
       <c r="E43" s="4"/>
     </row>
     <row r="44" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1300,9 +1283,9 @@
         <v>5</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D44" s="17"/>
+        <v>57</v>
+      </c>
+      <c r="D44" s="16"/>
       <c r="E44" s="4"/>
     </row>
     <row r="45" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1313,9 +1296,9 @@
         <v>7</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="D45" s="17"/>
+        <v>58</v>
+      </c>
+      <c r="D45" s="16"/>
       <c r="E45" s="4"/>
     </row>
     <row r="46" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1326,11 +1309,11 @@
         <v>10</v>
       </c>
       <c r="C46" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D46" s="16"/>
+      <c r="E46" s="4" t="s">
         <v>60</v>
-      </c>
-      <c r="D46" s="17"/>
-      <c r="E46" s="4" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1341,27 +1324,27 @@
         <v>5</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D47" s="17"/>
+        <v>53</v>
+      </c>
+      <c r="D47" s="16"/>
       <c r="E47" s="4"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="18" t="n">
+      <c r="A49" s="17" t="n">
         <v>46365</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C49" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D49" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D49" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:B47 C23 C2:C21 E22 C31:C47 C25:C29">
+  <conditionalFormatting sqref="A2:B47 C23 C2:C21 E22 C38:C47 C25:C27 C29:C36">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>$B2="F"</formula>
     </cfRule>

</xml_diff>